<commit_message>
nuovi utenti, corretto bug csv
</commit_message>
<xml_diff>
--- a/app/analysis/Questionnaire_results.xlsx
+++ b/app/analysis/Questionnaire_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -563,50 +563,50 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CS0</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>3.75</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E3" t="n">
-        <v>2.25</v>
+        <v>4.25</v>
       </c>
       <c r="F3" t="n">
-        <v>4</v>
+        <v>4.25</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>3.75</v>
       </c>
       <c r="H3" t="n">
-        <v>2.5</v>
+        <v>4.75</v>
       </c>
       <c r="I3" t="n">
-        <v>1.8</v>
+        <v>3.2</v>
       </c>
       <c r="J3" t="n">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="K3" t="n">
-        <v>2.2</v>
+        <v>4.2</v>
       </c>
       <c r="L3" t="n">
-        <v>2</v>
+        <v>3.8</v>
       </c>
       <c r="M3" t="n">
-        <v>2.8</v>
+        <v>4.4</v>
       </c>
       <c r="N3" t="n">
-        <v>3</v>
+        <v>3.8</v>
       </c>
       <c r="O3" t="n">
-        <v>1.8</v>
+        <v>5</v>
       </c>
       <c r="P3" t="n">
-        <v>1.4</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="4">
@@ -615,50 +615,50 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CS1</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3.5</v>
+        <v>3.75</v>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E4" t="n">
-        <v>4.5</v>
+        <v>4.25</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>4.25</v>
       </c>
       <c r="G4" t="n">
-        <v>3.25</v>
+        <v>3.75</v>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>4.75</v>
       </c>
       <c r="I4" t="n">
-        <v>4</v>
+        <v>2.6</v>
       </c>
       <c r="J4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M4" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="N4" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="O4" t="n">
         <v>2.4</v>
       </c>
-      <c r="K4" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="L4" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="M4" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="N4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O4" t="n">
-        <v>4</v>
-      </c>
       <c r="P4" t="n">
-        <v>3.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -667,50 +667,50 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2.75</v>
+        <v>3.75</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
-        <v>3.75</v>
+        <v>4.25</v>
       </c>
       <c r="F5" t="n">
-        <v>3.5</v>
+        <v>4.25</v>
       </c>
       <c r="G5" t="n">
-        <v>4</v>
+        <v>3.75</v>
       </c>
       <c r="H5" t="n">
-        <v>5</v>
+        <v>4.75</v>
       </c>
       <c r="I5" t="n">
-        <v>4.4</v>
+        <v>2.6</v>
       </c>
       <c r="J5" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="K5" t="n">
-        <v>4.2</v>
+        <v>2.8</v>
       </c>
       <c r="L5" t="n">
-        <v>2.8</v>
+        <v>3.8</v>
       </c>
       <c r="M5" t="n">
-        <v>3</v>
+        <v>3.6</v>
       </c>
       <c r="N5" t="n">
-        <v>2.2</v>
+        <v>3.8</v>
       </c>
       <c r="O5" t="n">
-        <v>4</v>
+        <v>2.4</v>
       </c>
       <c r="P5" t="n">
-        <v>3.6</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="6">
@@ -719,49 +719,829 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="L6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="N6" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="O6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="H7" t="n">
+        <v>4</v>
+      </c>
+      <c r="I7" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K7" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="L7" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M7" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="N7" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="O7" t="n">
+        <v>5</v>
+      </c>
+      <c r="P7" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="H8" t="n">
+        <v>4</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J8" t="n">
+        <v>5</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M8" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="N8" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="O8" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P8" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="H9" t="n">
+        <v>4</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L9" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M9" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="N9" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="O9" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P9" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="G10" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="L10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M10" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="N10" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="O10" t="n">
+        <v>5</v>
+      </c>
+      <c r="P10" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="G11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="I11" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J11" t="n">
+        <v>4</v>
+      </c>
+      <c r="K11" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="L11" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M11" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="N11" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="O11" t="n">
+        <v>5</v>
+      </c>
+      <c r="P11" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="I12" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J12" t="n">
+        <v>5</v>
+      </c>
+      <c r="K12" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L12" t="n">
+        <v>5</v>
+      </c>
+      <c r="M12" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="N12" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="O12" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P12" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D13" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="G13" t="n">
+        <v>3</v>
+      </c>
+      <c r="H13" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J13" t="n">
+        <v>4</v>
+      </c>
+      <c r="K13" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L13" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M13" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="N13" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="O13" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P13" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I14" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J14" t="n">
+        <v>5</v>
+      </c>
+      <c r="K14" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="L14" t="n">
+        <v>5</v>
+      </c>
+      <c r="M14" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="N14" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="O14" t="n">
+        <v>5</v>
+      </c>
+      <c r="P14" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4</v>
+      </c>
+      <c r="G15" t="n">
+        <v>3</v>
+      </c>
+      <c r="H15" t="n">
+        <v>4</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K15" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="L15" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M15" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="N15" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="O15" t="n">
+        <v>5</v>
+      </c>
+      <c r="P15" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4</v>
+      </c>
+      <c r="G16" t="n">
+        <v>3</v>
+      </c>
+      <c r="H16" t="n">
+        <v>4</v>
+      </c>
+      <c r="I16" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J16" t="n">
+        <v>5</v>
+      </c>
+      <c r="K16" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L16" t="n">
+        <v>5</v>
+      </c>
+      <c r="M16" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="N16" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="O16" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P16" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G17" t="n">
+        <v>3</v>
+      </c>
+      <c r="H17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I17" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K17" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L17" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M17" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="N17" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="O17" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P17" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="F18" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2</v>
+      </c>
+      <c r="H18" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="J18" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="K18" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="L18" t="n">
+        <v>2</v>
+      </c>
+      <c r="M18" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="N18" t="n">
+        <v>3</v>
+      </c>
+      <c r="O18" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="P18" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F19" t="n">
+        <v>3</v>
+      </c>
+      <c r="G19" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="H19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I19" t="n">
+        <v>4</v>
+      </c>
+      <c r="J19" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="K19" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="L19" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="M19" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="N19" t="n">
+        <v>2</v>
+      </c>
+      <c r="O19" t="n">
+        <v>4</v>
+      </c>
+      <c r="P19" t="n">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F20" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G20" t="n">
+        <v>4</v>
+      </c>
+      <c r="H20" t="n">
+        <v>5</v>
+      </c>
+      <c r="I20" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="J20" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="K20" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="M20" t="n">
+        <v>3</v>
+      </c>
+      <c r="N20" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="O20" t="n">
+        <v>4</v>
+      </c>
+      <c r="P20" t="n">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>II</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C21" t="n">
         <v>2.75</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D21" t="n">
         <v>2.75</v>
       </c>
-      <c r="E6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4</v>
-      </c>
-      <c r="G6" t="n">
+      <c r="E21" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" t="n">
         <v>1.75</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H21" t="n">
         <v>1.5</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I21" t="n">
         <v>2.8</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J21" t="n">
         <v>2.8</v>
       </c>
-      <c r="K6" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="L6" t="n">
+      <c r="K21" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="L21" t="n">
         <v>3</v>
       </c>
-      <c r="M6" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="N6" t="n">
+      <c r="M21" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="N21" t="n">
         <v>3</v>
       </c>
-      <c r="O6" t="n">
+      <c r="O21" t="n">
         <v>2.6</v>
       </c>
-      <c r="P6" t="n">
+      <c r="P21" t="n">
         <v>2.2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added new users; added new plot;
</commit_message>
<xml_diff>
--- a/app/analysis/Questionnaire_results.xlsx
+++ b/app/analysis/Questionnaire_results.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -692,59 +692,59 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>CS0</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>2.25</v>
+        <v>4</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>4</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>2</v>
+        <v>3.25</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>2.5</v>
+        <v>3.75</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>1.8</v>
+        <v>4.6</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>3.8</v>
+        <v>3.4</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>2.2</v>
+        <v>4</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>2</v>
+        <v>3.6</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>1.8</v>
+        <v>3.6</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>1.4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -752,51 +752,51 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>3.25</v>
+        <v>1</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>3.25</v>
+        <v>2</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>3.5</v>
+        <v>2.25</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>1.75</v>
+        <v>4</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>3.4</v>
+        <v>1.8</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>3</v>
+        <v>3.8</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>3</v>
+        <v>2.2</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>3.4</v>
+        <v>3</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>2.8</v>
+        <v>1.8</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
@@ -804,51 +804,51 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>2.5</v>
+        <v>3.25</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>2</v>
+        <v>3.25</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>4</v>
+        <v>1.75</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>4.25</v>
+        <v>4</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>4.6</v>
+        <v>3.4</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>4.8</v>
+        <v>3</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>4.4</v>
+        <v>3</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>4.8</v>
+        <v>3</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>4.2</v>
+        <v>2.8</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>4.2</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
@@ -856,103 +856,103 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>2.25</v>
+        <v>4</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>3.5</v>
+        <v>4.25</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>3.75</v>
+        <v>4.5</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>3</v>
+        <v>4.6</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>3</v>
+        <v>4.8</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>3.8</v>
+        <v>4.4</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>3.6</v>
+        <v>4.8</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>3</v>
+        <v>4.2</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>3.4</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>CS1</t>
+          <t>CS0</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="D9" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="F9" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G9" s="3" t="n">
-        <v>3.25</v>
-      </c>
       <c r="H9" s="3" t="n">
-        <v>3</v>
+        <v>3.75</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="L9" s="3" t="n">
         <v>3.6</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>1.6</v>
+        <v>3.4</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>3.8</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
@@ -960,51 +960,51 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="3" t="n">
         <v>3.25</v>
       </c>
-      <c r="D10" s="3" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>3</v>
-      </c>
       <c r="H10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="N10" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="I10" s="3" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="J10" s="3" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="K10" s="3" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="L10" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="M10" s="3" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="N10" s="3" t="n">
-        <v>2.4</v>
-      </c>
       <c r="O10" s="3" t="n">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>2.6</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
@@ -1012,103 +1012,103 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E11" s="3" t="n">
         <v>2.75</v>
       </c>
-      <c r="D11" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E11" s="3" t="n">
-        <v>2.5</v>
-      </c>
       <c r="F11" s="3" t="n">
-        <v>3.5</v>
+        <v>2.75</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>2.75</v>
+        <v>2</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>3.2</v>
+        <v>1.6</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>3.4</v>
+        <v>1.6</v>
       </c>
       <c r="K11" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="L11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" s="3" t="n">
         <v>2.6</v>
       </c>
-      <c r="L11" s="3" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="M11" s="3" t="n">
+      <c r="N11" s="3" t="n">
         <v>2.4</v>
       </c>
-      <c r="N11" s="3" t="n">
-        <v>3.2</v>
-      </c>
       <c r="O11" s="3" t="n">
-        <v>3.4</v>
+        <v>2.8</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>3.4</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>CS1</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>3.75</v>
+        <v>2.5</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>3.5</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>4</v>
+        <v>2.75</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>5</v>
+        <v>2.75</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>4.4</v>
+        <v>3.2</v>
       </c>
       <c r="J12" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="M12" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="N12" s="3" t="n">
         <v>3.2</v>
       </c>
-      <c r="K12" s="3" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="L12" s="3" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="M12" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="N12" s="3" t="n">
-        <v>2.2</v>
-      </c>
       <c r="O12" s="3" t="n">
-        <v>4</v>
+        <v>3.4</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -1116,150 +1116,306 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>2.5</v>
+        <v>2.75</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>4</v>
+        <v>3.75</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I13" s="3" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="M13" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="N13" s="3" t="n">
         <v>2.2</v>
       </c>
-      <c r="J13" s="3" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K13" s="3" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="L13" s="3" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="M13" s="3" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="N13" s="3" t="n">
-        <v>1.8</v>
-      </c>
       <c r="O13" s="3" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>2.4</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>4</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>2.8</v>
+        <v>2.2</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>2.8</v>
       </c>
       <c r="K14" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="M14" s="3" t="n">
         <v>3.2</v>
       </c>
-      <c r="L14" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="M14" s="3" t="n">
-        <v>3.8</v>
-      </c>
       <c r="N14" s="3" t="n">
-        <v>3</v>
+        <v>1.8</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>2.6</v>
+        <v>3.4</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="L15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M15" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="N15" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="O15" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="P15" s="3" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="L16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="M16" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="P16" s="3" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>II</t>
         </is>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="C17" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D17" s="3" t="n">
         <v>1.25</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E17" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="3" t="n">
+      <c r="F17" s="3" t="n">
         <v>1.25</v>
       </c>
-      <c r="G15" s="3" t="n">
+      <c r="G17" s="3" t="n">
         <v>1.25</v>
       </c>
-      <c r="H15" s="3" t="n">
+      <c r="H17" s="3" t="n">
         <v>1.5</v>
       </c>
-      <c r="I15" s="3" t="n">
+      <c r="I17" s="3" t="n">
         <v>2.2</v>
       </c>
-      <c r="J15" s="3" t="n">
+      <c r="J17" s="3" t="n">
         <v>1.8</v>
       </c>
-      <c r="K15" s="3" t="n">
+      <c r="K17" s="3" t="n">
         <v>1.6</v>
       </c>
-      <c r="L15" s="3" t="n">
+      <c r="L17" s="3" t="n">
         <v>1.4</v>
       </c>
-      <c r="M15" s="3" t="n">
+      <c r="M17" s="3" t="n">
         <v>1.6</v>
       </c>
-      <c r="N15" s="3" t="n">
+      <c r="N17" s="3" t="n">
         <v>1.8</v>
       </c>
-      <c r="O15" s="3" t="n">
+      <c r="O17" s="3" t="n">
         <v>1.2</v>
       </c>
-      <c r="P15" s="3" t="n">
+      <c r="P17" s="3" t="n">
         <v>1.6</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="L18" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="M18" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="O18" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="P18" s="3" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>